<commit_message>
Update unpaid repasse values in Controle spreadsheet and HTML report based on the current pricing table (New total: R$ 26,690.80)
</commit_message>
<xml_diff>
--- a/MDUs_Faturados_Historico_Controle.xlsx
+++ b/MDUs_Faturados_Historico_Controle.xlsx
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>520</v>
+        <v>551.2</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>520</v>
+        <v>551.2</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>520</v>
+        <v>551.2</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -719,7 +719,7 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>1040</v>
+        <v>996.4</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>520</v>
+        <v>551.2</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -841,7 +841,7 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>520</v>
+        <v>551.2</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -902,7 +902,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>520</v>
+        <v>551.2</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>520</v>
+        <v>551.2</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1024,7 +1024,7 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>520</v>
+        <v>551.2</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1085,7 +1085,7 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>520</v>
+        <v>551.2</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -1146,7 +1146,7 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>520</v>
+        <v>551.2</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -1207,7 +1207,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>520</v>
+        <v>551.2</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -1268,7 +1268,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>520</v>
+        <v>551.2</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -1329,7 +1329,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>520</v>
+        <v>996.4</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -1390,7 +1390,7 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>520</v>
+        <v>996.4</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
@@ -1451,7 +1451,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>520</v>
+        <v>996.4</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
@@ -1512,7 +1512,7 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>940</v>
+        <v>720.8</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="L19" t="n">
-        <v>620</v>
+        <v>551.2</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
@@ -1634,7 +1634,7 @@
         </is>
       </c>
       <c r="L20" t="n">
-        <v>520</v>
+        <v>551.2</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
@@ -1695,7 +1695,7 @@
         </is>
       </c>
       <c r="L21" t="n">
-        <v>780</v>
+        <v>720.8</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
@@ -1756,7 +1756,7 @@
         </is>
       </c>
       <c r="L22" t="n">
-        <v>520</v>
+        <v>551.2</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
@@ -1817,7 +1817,7 @@
         </is>
       </c>
       <c r="L23" t="n">
-        <v>620</v>
+        <v>551.2</v>
       </c>
       <c r="M23" t="inlineStr">
         <is>
@@ -1878,7 +1878,7 @@
         </is>
       </c>
       <c r="L24" t="n">
-        <v>520</v>
+        <v>551.2</v>
       </c>
       <c r="M24" t="inlineStr">
         <is>
@@ -1939,7 +1939,7 @@
         </is>
       </c>
       <c r="L25" t="n">
-        <v>520</v>
+        <v>551.2</v>
       </c>
       <c r="M25" t="inlineStr">
         <is>
@@ -2000,7 +2000,7 @@
         </is>
       </c>
       <c r="L26" t="n">
-        <v>680</v>
+        <v>720.8</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>
@@ -2061,7 +2061,7 @@
         </is>
       </c>
       <c r="L27" t="n">
-        <v>1040</v>
+        <v>720.8</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
@@ -2122,7 +2122,7 @@
         </is>
       </c>
       <c r="L28" t="n">
-        <v>1040</v>
+        <v>720.8</v>
       </c>
       <c r="M28" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
         </is>
       </c>
       <c r="L29" t="n">
-        <v>1040</v>
+        <v>720.8</v>
       </c>
       <c r="M29" t="inlineStr">
         <is>
@@ -2244,7 +2244,7 @@
         </is>
       </c>
       <c r="L30" t="n">
-        <v>1040</v>
+        <v>720.8</v>
       </c>
       <c r="M30" t="inlineStr">
         <is>
@@ -2305,7 +2305,7 @@
         </is>
       </c>
       <c r="L31" t="n">
-        <v>520</v>
+        <v>551.2</v>
       </c>
       <c r="M31" t="inlineStr">
         <is>
@@ -2366,7 +2366,7 @@
         </is>
       </c>
       <c r="L32" t="n">
-        <v>520</v>
+        <v>551.2</v>
       </c>
       <c r="M32" t="inlineStr">
         <is>
@@ -2427,7 +2427,7 @@
         </is>
       </c>
       <c r="L33" t="n">
-        <v>620</v>
+        <v>551.2</v>
       </c>
       <c r="M33" t="inlineStr">
         <is>
@@ -2488,7 +2488,7 @@
         </is>
       </c>
       <c r="L34" t="n">
-        <v>620</v>
+        <v>551.2</v>
       </c>
       <c r="M34" t="inlineStr">
         <is>
@@ -2549,7 +2549,7 @@
         </is>
       </c>
       <c r="L35" t="n">
-        <v>620</v>
+        <v>551.2</v>
       </c>
       <c r="M35" t="inlineStr">
         <is>
@@ -2610,7 +2610,7 @@
         </is>
       </c>
       <c r="L36" t="n">
-        <v>520</v>
+        <v>551.2</v>
       </c>
       <c r="M36" t="inlineStr">
         <is>
@@ -2671,7 +2671,7 @@
         </is>
       </c>
       <c r="L37" t="n">
-        <v>780</v>
+        <v>720.8</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
@@ -2732,7 +2732,7 @@
         </is>
       </c>
       <c r="L38" t="n">
-        <v>780</v>
+        <v>720.8</v>
       </c>
       <c r="M38" t="inlineStr">
         <is>
@@ -2793,7 +2793,7 @@
         </is>
       </c>
       <c r="L39" t="n">
-        <v>780</v>
+        <v>720.8</v>
       </c>
       <c r="M39" t="inlineStr">
         <is>
@@ -2854,7 +2854,7 @@
         </is>
       </c>
       <c r="L40" t="n">
-        <v>680</v>
+        <v>996.4</v>
       </c>
       <c r="M40" t="inlineStr">
         <is>
@@ -2915,7 +2915,7 @@
         </is>
       </c>
       <c r="L41" t="n">
-        <v>780</v>
+        <v>720.8</v>
       </c>
       <c r="M41" t="inlineStr">
         <is>
@@ -2976,7 +2976,7 @@
         </is>
       </c>
       <c r="L42" t="n">
-        <v>520</v>
+        <v>551.2</v>
       </c>
       <c r="M42" t="inlineStr">
         <is>

</xml_diff>